<commit_message>
+ add new menuitem convert
</commit_message>
<xml_diff>
--- a/SimpleMenuTemplate.xlsx
+++ b/SimpleMenuTemplate.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Nan_Dev\ZiiPOSMenuConvertor\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nan_Dev\ZiiPOSMenuConvertor\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36549392-0A32-44AC-9C19-32AC6A2C33D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7F28762-D32A-44AC-9734-4A18F3279DB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4068" yWindow="1848" windowWidth="17280" windowHeight="8832" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="54">
   <si>
     <t>ItemCode</t>
   </si>
@@ -152,6 +152,48 @@
   </si>
   <si>
     <t>A002</t>
+  </si>
+  <si>
+    <t>A033</t>
+  </si>
+  <si>
+    <t>Drink</t>
+  </si>
+  <si>
+    <t>Latte</t>
+  </si>
+  <si>
+    <t>Coffe</t>
+  </si>
+  <si>
+    <t>Small</t>
+  </si>
+  <si>
+    <t>Mid</t>
+  </si>
+  <si>
+    <t>Large</t>
+  </si>
+  <si>
+    <t>Ex.Large</t>
+  </si>
+  <si>
+    <t>A050</t>
+  </si>
+  <si>
+    <t>Misc</t>
+  </si>
+  <si>
+    <t>Others</t>
+  </si>
+  <si>
+    <t>C090</t>
+  </si>
+  <si>
+    <t>Candy KG</t>
+  </si>
+  <si>
+    <t>Candy</t>
   </si>
 </sst>
 </file>
@@ -216,9 +258,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -256,7 +298,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -362,7 +404,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -504,7 +546,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -512,28 +554,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AH3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:AH6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.6640625" customWidth="1"/>
-    <col min="2" max="2" width="21.5546875" customWidth="1"/>
-    <col min="3" max="3" width="18.6640625" customWidth="1"/>
-    <col min="4" max="4" width="20.109375" customWidth="1"/>
-    <col min="5" max="5" width="22.44140625" customWidth="1"/>
-    <col min="6" max="6" width="20.6640625" customWidth="1"/>
-    <col min="7" max="11" width="10.6640625" customWidth="1"/>
-    <col min="12" max="12" width="16.5546875" customWidth="1"/>
-    <col min="13" max="20" width="16.6640625" customWidth="1"/>
-    <col min="21" max="24" width="18.6640625" customWidth="1"/>
-    <col min="25" max="25" width="12.6640625" customWidth="1"/>
-    <col min="26" max="27" width="10.6640625" customWidth="1"/>
-    <col min="28" max="28" width="12.6640625" customWidth="1"/>
-    <col min="29" max="29" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="31" max="34" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" customWidth="1"/>
+    <col min="4" max="4" width="20.140625" customWidth="1"/>
+    <col min="5" max="5" width="22.42578125" customWidth="1"/>
+    <col min="6" max="6" width="20.7109375" customWidth="1"/>
+    <col min="7" max="11" width="10.7109375" customWidth="1"/>
+    <col min="12" max="12" width="16.5703125" customWidth="1"/>
+    <col min="13" max="13" width="12.7109375" customWidth="1"/>
+    <col min="14" max="17" width="18.7109375" customWidth="1"/>
+    <col min="18" max="25" width="16.7109375" customWidth="1"/>
+    <col min="26" max="26" width="12.7109375" customWidth="1"/>
+    <col min="27" max="28" width="10.7109375" customWidth="1"/>
+    <col min="29" max="29" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="31" max="34" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -571,52 +613,52 @@
         <v>19</v>
       </c>
       <c r="M1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="R1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="U1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>27</v>
       </c>
       <c r="AC1" t="s">
         <v>32</v>
@@ -637,7 +679,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>28</v>
       </c>
@@ -665,19 +707,7 @@
       <c r="L2">
         <v>10</v>
       </c>
-      <c r="M2">
-        <v>0</v>
-      </c>
-      <c r="N2">
-        <v>0</v>
-      </c>
-      <c r="O2">
-        <v>0</v>
-      </c>
-      <c r="P2">
-        <v>0</v>
-      </c>
-      <c r="Q2">
+      <c r="M2" t="b">
         <v>0</v>
       </c>
       <c r="R2">
@@ -689,7 +719,19 @@
       <c r="T2">
         <v>0</v>
       </c>
-      <c r="Y2" t="b">
+      <c r="U2">
+        <v>0</v>
+      </c>
+      <c r="V2">
+        <v>0</v>
+      </c>
+      <c r="W2">
+        <v>0</v>
+      </c>
+      <c r="X2">
+        <v>0</v>
+      </c>
+      <c r="Y2">
         <v>0</v>
       </c>
       <c r="Z2" t="b">
@@ -720,7 +762,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>39</v>
       </c>
@@ -748,19 +790,7 @@
       <c r="L3">
         <v>10</v>
       </c>
-      <c r="M3">
-        <v>0</v>
-      </c>
-      <c r="N3">
-        <v>0</v>
-      </c>
-      <c r="O3">
-        <v>0</v>
-      </c>
-      <c r="P3">
-        <v>0</v>
-      </c>
-      <c r="Q3">
+      <c r="M3" t="b">
         <v>0</v>
       </c>
       <c r="R3">
@@ -772,7 +802,19 @@
       <c r="T3">
         <v>0</v>
       </c>
-      <c r="Y3" t="b">
+      <c r="U3">
+        <v>0</v>
+      </c>
+      <c r="V3">
+        <v>0</v>
+      </c>
+      <c r="W3">
+        <v>0</v>
+      </c>
+      <c r="X3">
+        <v>0</v>
+      </c>
+      <c r="Y3">
         <v>0</v>
       </c>
       <c r="Z3" t="b">
@@ -800,6 +842,264 @@
         <v>0</v>
       </c>
       <c r="AH3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" t="s">
+        <v>42</v>
+      </c>
+      <c r="F4" t="s">
+        <v>43</v>
+      </c>
+      <c r="G4" t="s">
+        <v>41</v>
+      </c>
+      <c r="H4">
+        <v>4</v>
+      </c>
+      <c r="I4">
+        <v>4.5</v>
+      </c>
+      <c r="J4">
+        <v>5</v>
+      </c>
+      <c r="K4">
+        <v>5.5</v>
+      </c>
+      <c r="L4">
+        <v>10</v>
+      </c>
+      <c r="M4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N4" t="s">
+        <v>44</v>
+      </c>
+      <c r="O4" t="s">
+        <v>45</v>
+      </c>
+      <c r="P4" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>47</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <v>0</v>
+      </c>
+      <c r="U4">
+        <v>0</v>
+      </c>
+      <c r="V4">
+        <v>0</v>
+      </c>
+      <c r="W4">
+        <v>0</v>
+      </c>
+      <c r="X4">
+        <v>0</v>
+      </c>
+      <c r="Y4">
+        <v>0</v>
+      </c>
+      <c r="Z4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB4" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AE4">
+        <v>0</v>
+      </c>
+      <c r="AF4">
+        <v>0</v>
+      </c>
+      <c r="AG4">
+        <v>0</v>
+      </c>
+      <c r="AH4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G5" t="s">
+        <v>50</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>10</v>
+      </c>
+      <c r="M5" t="b">
+        <v>0</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+      <c r="T5">
+        <v>0</v>
+      </c>
+      <c r="U5">
+        <v>0</v>
+      </c>
+      <c r="V5">
+        <v>0</v>
+      </c>
+      <c r="W5">
+        <v>0</v>
+      </c>
+      <c r="X5">
+        <v>0</v>
+      </c>
+      <c r="Y5">
+        <v>0</v>
+      </c>
+      <c r="Z5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="b">
+        <v>0</v>
+      </c>
+      <c r="AB5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AE5">
+        <v>0</v>
+      </c>
+      <c r="AF5">
+        <v>0</v>
+      </c>
+      <c r="AG5">
+        <v>0</v>
+      </c>
+      <c r="AH5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H6">
+        <v>5</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>10</v>
+      </c>
+      <c r="M6" t="b">
+        <v>0</v>
+      </c>
+      <c r="R6">
+        <v>0</v>
+      </c>
+      <c r="S6">
+        <v>0</v>
+      </c>
+      <c r="T6">
+        <v>0</v>
+      </c>
+      <c r="U6">
+        <v>0</v>
+      </c>
+      <c r="V6">
+        <v>0</v>
+      </c>
+      <c r="W6">
+        <v>0</v>
+      </c>
+      <c r="X6">
+        <v>0</v>
+      </c>
+      <c r="Y6">
+        <v>0</v>
+      </c>
+      <c r="Z6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB6" t="b">
+        <v>0</v>
+      </c>
+      <c r="AC6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AE6">
+        <v>0</v>
+      </c>
+      <c r="AF6">
+        <v>0</v>
+      </c>
+      <c r="AG6">
         <v>0</v>
       </c>
     </row>

</xml_diff>